<commit_message>
Add requirements.txt; run reorder before load in main
Pin pandas/openpyxl/scipy for a dedicated project venv. main.py now
reorders the workbook by Pond ID first, then loads the reordered copy.
</commit_message>
<xml_diff>
--- a/data/Outcome Evaluation Phase 2 Data_Cleaned And Anonymized.reordered.xlsx
+++ b/data/Outcome Evaluation Phase 2 Data_Cleaned And Anonymized.reordered.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OOR Events" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="OOR Events" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Exclude no-follow-up OOR events from resolution rate
resolved=None events (no follow-up in the 5-day window) are now excluded
from the resolution rate in both analyze_oor_events and the pie, with a
clean bool cast keeping mean/sum well-defined. Add a with_followup column,
document the >5-day same-pond gap assumption, and restore sheet cross-checks.
</commit_message>
<xml_diff>
--- a/data/Outcome Evaluation Phase 2 Data_Cleaned And Anonymized.reordered.xlsx
+++ b/data/Outcome Evaluation Phase 2 Data_Cleaned And Anonymized.reordered.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="OOR Events" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OOR Events" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Add OOR resolution rate by parameter
oor_resolution_by_parameter + describe_resolution_by_parameter report the
Day-3 resolution rate overall and per OOR parameter (DO/pH/Ammonia) for
each group; multi-parameter events count toward each parameter. Wired into
main. Completes the "proportion resolved (overall and by parameter)"
descriptive-stats bullet.
</commit_message>
<xml_diff>
--- a/data/Outcome Evaluation Phase 2 Data_Cleaned And Anonymized.reordered.xlsx
+++ b/data/Outcome Evaluation Phase 2 Data_Cleaned And Anonymized.reordered.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OOR Events" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="OOR Events" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>